<commit_message>
[Feat] DataManager,NPCManager,QuestManager 작성, 편지함 UI 연결 중
NPC,Quest 데이터 관리 시스템 작성
- Manager : 관리 로직 담당
- Data : 데이터 보유, 데이터 변경 로직 담당
- NPC/Quest: 원본 데이터 래핑 담당

DataManager: 원본 데이터 Loader 생성.

*주의사항: 테스트 시에 하이어라키에 Manager 오브젝트를 생성해두는 편이 좋음(초기화 순서 문제)

npc/quest와 편지함 UI 간 연결이 더 필요함.
퀘스트 수락 거절 시 효과 부분에 대한 로직 추가 필요.
</commit_message>
<xml_diff>
--- a/Excel2JSON(win-x64)/excel_files/Enum.xlsx
+++ b/Excel2JSON(win-x64)/excel_files/Enum.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28803"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3C6568D-E588-4658-9AB9-AB50E80B078A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0AFF9C9-DD25-423E-A9D3-AEBEA930C5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Enum" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Grade</t>
   </si>
@@ -48,9 +48,6 @@
     <t>Region</t>
   </si>
   <si>
-    <t>all</t>
-  </si>
-  <si>
     <t>gangwon</t>
   </si>
   <si>
@@ -139,6 +136,42 @@
   </si>
   <si>
     <t>high</t>
+  </si>
+  <si>
+    <t>Route</t>
+  </si>
+  <si>
+    <t>gather</t>
+  </si>
+  <si>
+    <t>NPC</t>
+  </si>
+  <si>
+    <t>cook</t>
+  </si>
+  <si>
+    <t>CookingTool</t>
+  </si>
+  <si>
+    <t>doma</t>
+  </si>
+  <si>
+    <t>julgu</t>
+  </si>
+  <si>
+    <t>matdol</t>
+  </si>
+  <si>
+    <t>gamasot</t>
+  </si>
+  <si>
+    <t>sotdduggung</t>
+  </si>
+  <si>
+    <t>mixingbowl</t>
+  </si>
+  <si>
+    <t>dish</t>
   </si>
 </sst>
 </file>
@@ -157,7 +190,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -168,7 +201,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -176,174 +209,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -677,185 +549,171 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O6"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34787D26-712A-4F94-BDB7-B6CFEB19172B}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:14" ht="16.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="3"/>
     </row>
-    <row r="2" spans="1:15">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:14" ht="16.5">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="6" t="s">
+    </row>
+    <row r="3" spans="1:14" ht="16.5">
+      <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="B3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="3" spans="1:15">
-      <c r="A3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="5" t="s">
+    <row r="4" spans="1:14" ht="16.5">
+      <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="6"/>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="4" spans="1:15">
-      <c r="A4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="5" t="s">
+    <row r="5" spans="1:14" ht="16.5">
+      <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="6"/>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="5" spans="1:15">
-      <c r="A5" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="5" t="s">
+    <row r="6" spans="1:14" ht="16.5">
+      <c r="A6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="6"/>
+      <c r="B6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="6" spans="1:15">
-      <c r="A6" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="8" t="s">
+    <row r="7" spans="1:14" ht="16.5">
+      <c r="A7" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="9"/>
+      <c r="B7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="16.5">
+      <c r="A8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[Feat] Popup sortingOrder, JSON Data 최신화
Enum 이름 변경으로 인해 몇몇 변수에서 타입 에러가 나는 부분 수정함.

ForestGatheringManager 58번째줄에서 사용하고 있는 메서드는 DataLoader_Gathering에 추가한 메서드라서, Data 최신화 과정에서 삭제됨.
</commit_message>
<xml_diff>
--- a/Excel2JSON(win-x64)/excel_files/Enum.xlsx
+++ b/Excel2JSON(win-x64)/excel_files/Enum.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28803"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28816"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0AFF9C9-DD25-423E-A9D3-AEBEA930C5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0AEBE9A2-578C-418E-AA8D-E6CB244A63AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,9 +31,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
-  <si>
-    <t>Grade</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
+  <si>
+    <t>GradeType</t>
   </si>
   <si>
     <t>common</t>
@@ -45,7 +45,7 @@
     <t>legendary</t>
   </si>
   <si>
-    <t>Region</t>
+    <t>RegionType</t>
   </si>
   <si>
     <t>gangwon</t>
@@ -87,7 +87,7 @@
     <t>northPyongan</t>
   </si>
   <si>
-    <t>Biome</t>
+    <t>BiomeType</t>
   </si>
   <si>
     <t>forest</t>
@@ -96,7 +96,7 @@
     <t>sea</t>
   </si>
   <si>
-    <t>Foreign</t>
+    <t>ForeignType</t>
   </si>
   <si>
     <t>japan</t>
@@ -108,7 +108,7 @@
     <t>none</t>
   </si>
   <si>
-    <t>Season</t>
+    <t>SeasonType</t>
   </si>
   <si>
     <t>spring</t>
@@ -123,7 +123,7 @@
     <t>winter</t>
   </si>
   <si>
-    <t>Chance</t>
+    <t>ChanceType</t>
   </si>
   <si>
     <t>veryLow</t>
@@ -138,7 +138,7 @@
     <t>high</t>
   </si>
   <si>
-    <t>Route</t>
+    <t>RouteType</t>
   </si>
   <si>
     <t>gather</t>
@@ -150,7 +150,7 @@
     <t>cook</t>
   </si>
   <si>
-    <t>CookingTool</t>
+    <t>CookingToolType</t>
   </si>
   <si>
     <t>doma</t>
@@ -172,6 +172,12 @@
   </si>
   <si>
     <t>dish</t>
+  </si>
+  <si>
+    <t>ItemType</t>
+  </si>
+  <si>
+    <t>ingredient</t>
   </si>
 </sst>
 </file>
@@ -553,7 +559,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:14" ht="16.5">
@@ -713,6 +719,17 @@
         <v>46</v>
       </c>
     </row>
+    <row r="9" spans="1:14" ht="15.75" customHeight="1">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>

</xml_diff>